<commit_message>
Addition of the maximum derivative
</commit_message>
<xml_diff>
--- a/Resumo_Features.xlsx
+++ b/Resumo_Features.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="32" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="53" uniqueCount="24">
   <si>
     <t>Feature</t>
   </si>
@@ -64,6 +64,27 @@
   </si>
   <si>
     <t>MediaImportancia</t>
+  </si>
+  <si>
+    <t>dPMax</t>
+  </si>
+  <si>
+    <t>TRelativoVmax</t>
+  </si>
+  <si>
+    <t>dVMax</t>
+  </si>
+  <si>
+    <t>TRelativoRmax</t>
+  </si>
+  <si>
+    <t>TRelativoImax</t>
+  </si>
+  <si>
+    <t>dIMax</t>
+  </si>
+  <si>
+    <t>dRMax</t>
   </si>
 </sst>
 </file>
@@ -109,7 +130,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="true"/>
@@ -133,10 +154,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C2" s="0">
-        <v>120.08943341239036</v>
+        <v>108.0596226437922</v>
       </c>
     </row>
     <row r="3">
@@ -144,10 +165,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C3" s="0">
-        <v>98.080145590354178</v>
+        <v>96.845767656440373</v>
       </c>
     </row>
     <row r="4">
@@ -155,10 +176,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C4" s="0">
-        <v>97.363584272403614</v>
+        <v>90.12795046033709</v>
       </c>
     </row>
     <row r="5">
@@ -166,120 +187,164 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C5" s="0">
-        <v>71.524427991982023</v>
+        <v>54.329677109189426</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B6" s="0">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C6" s="0">
-        <v>29.490393665061386</v>
+        <v>29.819087588194776</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B7" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="0">
-        <v>4.4652233308051059</v>
+        <v>23.79217282142066</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C8" s="0">
-        <v>4.1358701787901566</v>
+        <v>15.910545669563215</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B9" s="0">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C9" s="0">
-        <v>3.6507229883820318</v>
+        <v>7.932227769218188</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" s="0">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="C10" s="0">
-        <v>3.0897611803632397</v>
+        <v>3.0366996195952582</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B11" s="0">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="C11" s="0">
-        <v>2.8960216992203516</v>
+        <v>2.828140390161979</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B12" s="0">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C12" s="0">
-        <v>2.8742669041092341</v>
+        <v>2.6418647744546342</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B13" s="0">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C13" s="0">
-        <v>2.2303933563781801</v>
+        <v>2.3526122298680185</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B14" s="0">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C14" s="0">
-        <v>1.8201412429426889</v>
+        <v>2.1587260700394721</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B15" s="0">
+        <v>3</v>
+      </c>
+      <c r="C15" s="0">
+        <v>2.0331199974531526</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="0">
+        <v>3</v>
+      </c>
+      <c r="C16" s="0">
+        <v>2.0101373362375941</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="0">
+        <v>6</v>
+      </c>
+      <c r="C17" s="0">
+        <v>1.4551405673291578</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="0">
+        <v>2</v>
+      </c>
+      <c r="C18" s="0">
+        <v>0.071482267483068518</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="0">
         <v>1</v>
       </c>
-      <c r="C15" s="0">
-        <v>1.7390624950183908</v>
+      <c r="C19" s="0">
+        <v>0.039044287980524041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>